<commit_message>
Adding live test of load cell
</commit_message>
<xml_diff>
--- a/scripts/aquire_data/test_angles.xlsx
+++ b/scripts/aquire_data/test_angles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wind Turbine PC\Documents\Kyle\Github\BladeAccelerations\scripts\aquire_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21917773-C29D-4929-B00E-5544404FA994}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{736F1791-3334-4C29-B9FE-48ABCE960E0A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8DFE66DF-68FE-4367-A893-D93A9533A967}"/>
   </bookViews>
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564B26A9-E64A-4C57-86B1-B51A64E062CD}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -420,27 +420,127 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2">
-        <v>-10</v>
+        <v>-180</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3">
-        <v>-5</v>
+        <v>-165</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4">
-        <v>0</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5">
-        <v>5</v>
+        <v>-135</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6">
-        <v>10</v>
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10">
+        <v>-60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11">
+        <v>-45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13">
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changing default input for tests
</commit_message>
<xml_diff>
--- a/scripts/aquire_data/test_angles.xlsx
+++ b/scripts/aquire_data/test_angles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wind Turbine PC\Documents\Kyle\Github\BladeAccelerations\scripts\aquire_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{736F1791-3334-4C29-B9FE-48ABCE960E0A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F0F8EB-E070-495F-B80C-77453C146A76}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8DFE66DF-68FE-4367-A893-D93A9533A967}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8DFE66DF-68FE-4367-A893-D93A9533A967}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564B26A9-E64A-4C57-86B1-B51A64E062CD}">
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -420,92 +420,92 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2">
-        <v>-180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3">
-        <v>-165</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4">
-        <v>-150</v>
+        <v>-70</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5">
-        <v>-135</v>
+        <v>-60</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6">
-        <v>-120</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7">
-        <v>-105</v>
+        <v>-40</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8">
-        <v>-90</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9">
-        <v>-75</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10">
-        <v>-60</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11">
-        <v>-45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12">
-        <v>-30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13">
-        <v>-15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:1">
@@ -515,32 +515,127 @@
     </row>
     <row r="21" spans="1:1">
       <c r="A21">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22">
-        <v>120</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23">
-        <v>135</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24">
-        <v>150</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25">
-        <v>165</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35">
         <v>180</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45">
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>